<commit_message>
Update project management documents
</commit_message>
<xml_diff>
--- a/project_management/Defect_Tracker Template_v0.1.xlsx
+++ b/project_management/Defect_Tracker Template_v0.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://infosystechnologies-my.sharepoint.com/personal/kamaljeet_kaur01_ad_infosys_com1/Documents/Infosys/CC/Events/Oct 2021 - Mar 2022/CC2.0/Internship/Jan-Apr 2022/Artifacts/internship/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b15b4f3444aaab9/Desktop/INFOSYS/ai-response-validation-system/project_management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1529751A-99C4-4233-8104-CEB3E356847C}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7F2B3EB-1E6D-418A-8DB4-1B3A95BE19AF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Defects" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>Sl No</t>
   </si>
@@ -69,6 +69,24 @@
   </si>
   <si>
     <t>Status(Open/Closed)</t>
+  </si>
+  <si>
+    <t>Vinod</t>
+  </si>
+  <si>
+    <t>Validation submission was blocked when no reference answer or source document was provided</t>
+  </si>
+  <si>
+    <t>Sprint 1</t>
+  </si>
+  <si>
+    <t>Updated the validation flow to allow evidence-based evaluation without a reference answer</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>Fixed and tested successfully</t>
   </si>
 </sst>
 </file>
@@ -209,9 +227,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -249,9 +267,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -284,26 +302,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -336,26 +337,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -530,21 +514,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K20"/>
-  <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="17.5546875" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="42.140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="42.109375" style="4" customWidth="1"/>
     <col min="5" max="5" width="16" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="21.85546875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="16.85546875" style="4" customWidth="1"/>
-    <col min="12" max="16384" width="17.5703125" style="4"/>
+    <col min="6" max="6" width="12.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="21.88671875" style="4" customWidth="1"/>
+    <col min="11" max="11" width="16.88671875" style="4" customWidth="1"/>
+    <col min="12" max="16384" width="17.5546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -579,20 +563,38 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
+    <row r="2" spans="1:11" ht="78" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="D2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="J2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -605,7 +607,7 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -618,7 +620,7 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -631,7 +633,7 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -644,7 +646,7 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="5"/>
       <c r="C7" s="5"/>
@@ -657,7 +659,7 @@
       <c r="J7" s="3"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -670,7 +672,7 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="5"/>
       <c r="C9" s="5"/>
@@ -683,7 +685,7 @@
       <c r="J9" s="3"/>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -696,7 +698,7 @@
       <c r="J10" s="3"/>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -709,7 +711,7 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
     </row>
-    <row r="12" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -722,7 +724,7 @@
       <c r="J12" s="3"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -735,7 +737,7 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -748,7 +750,7 @@
       <c r="J14" s="3"/>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -761,7 +763,7 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -774,7 +776,7 @@
       <c r="J16" s="3"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -787,7 +789,7 @@
       <c r="J17" s="3"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -800,7 +802,7 @@
       <c r="J18" s="3"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -813,7 +815,7 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
     </row>
-    <row r="20" spans="1:11" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -849,29 +851,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>14</v>
       </c>
@@ -883,6 +885,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1014,12 +1022,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1030,6 +1032,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1047,15 +1058,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update Milestone 2 project management documents
</commit_message>
<xml_diff>
--- a/project_management/Defect_Tracker Template_v0.1.xlsx
+++ b/project_management/Defect_Tracker Template_v0.1.xlsx
@@ -224,6 +224,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -885,12 +889,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F50FC49184C87E449886FB52439922C9" ma:contentTypeVersion="2" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f85b7e58c3d8889ba0673e7b34a193a6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b67b99c0-208c-4860-83e0-51466af787c4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d43477c1ade21a66d9a75ba2d5aa042" ns2:_="">
     <xsd:import namespace="b67b99c0-208c-4860-83e0-51466af787c4"/>
@@ -1022,6 +1020,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1032,15 +1036,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{191CB444-B9BF-4C91-94BD-600524521497}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1058,6 +1053,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>

</xml_diff>